<commit_message>
test: Use UTC time
</commit_message>
<xml_diff>
--- a/test/snap/readme.snap.xlsx
+++ b/test/snap/readme.snap.xlsx
@@ -336,7 +336,7 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <v>43102.642245</v>
+        <v>43102.573495</v>
       </c>
     </row>
     <row r="9">
@@ -346,7 +346,7 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <v>43102.642245</v>
+        <v>43102.573495</v>
       </c>
     </row>
     <row r="10">
@@ -356,7 +356,7 @@
         </is>
       </c>
       <c r="B10" s="1">
-        <v>43102.642245</v>
+        <v>43102.573495</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix styles.xml for Open XML schema
Emit a complete styleSheet part per SpreadsheetML: cellXfs with numFmtId,
fillId, borderId and xfId; required cellStyleXfs and cellStyles sections;
CT_Font children in schema order with boolean val attributes; and 8-digit
ARGB rgb values (ST_UnsignedIntHex) for solid fills.
</commit_message>
<xml_diff>
--- a/test/snap/readme.snap.xlsx
+++ b/test/snap/readme.snap.xlsx
@@ -22,9 +22,9 @@
       <name val="Calibri"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <b/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,12 +38,18 @@
   <borders count="1">
     <border/>
   </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
   <cellXfs count="4">
     <xf fontId="0" applyFont="1"/>
     <xf numFmtId="164" applyNumberFormat="1"/>
     <xf numFmtId="165" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" applyFont="1"/>
   </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
 </styleSheet>
 </file>
 

</xml_diff>